<commit_message>
try to create a new heatmap method on sipak
</commit_message>
<xml_diff>
--- a/results/excel_reports/resnet50_vgg16_black.xlsx
+++ b/results/excel_reports/resnet50_vgg16_black.xlsx
@@ -199,12 +199,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$2:$U$2</f>
+              <f>'Data'!$B$2:$V$2</f>
             </numRef>
           </val>
         </ser>
@@ -231,12 +231,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$3:$U$3</f>
+              <f>'Data'!$B$3:$V$3</f>
             </numRef>
           </val>
         </ser>
@@ -263,12 +263,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$4:$U$4</f>
+              <f>'Data'!$B$4:$V$4</f>
             </numRef>
           </val>
         </ser>
@@ -295,12 +295,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$5:$U$5</f>
+              <f>'Data'!$B$5:$V$5</f>
             </numRef>
           </val>
         </ser>
@@ -327,12 +327,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$6:$U$6</f>
+              <f>'Data'!$B$6:$V$6</f>
             </numRef>
           </val>
         </ser>
@@ -359,12 +359,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$7:$U$7</f>
+              <f>'Data'!$B$7:$V$7</f>
             </numRef>
           </val>
         </ser>
@@ -391,12 +391,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$8:$U$8</f>
+              <f>'Data'!$B$8:$V$8</f>
             </numRef>
           </val>
         </ser>
@@ -423,12 +423,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$9:$U$9</f>
+              <f>'Data'!$B$9:$V$9</f>
             </numRef>
           </val>
         </ser>
@@ -455,12 +455,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$10:$U$10</f>
+              <f>'Data'!$B$10:$V$10</f>
             </numRef>
           </val>
         </ser>
@@ -487,12 +487,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$11:$U$11</f>
+              <f>'Data'!$B$11:$V$11</f>
             </numRef>
           </val>
         </ser>
@@ -519,12 +519,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$12:$U$12</f>
+              <f>'Data'!$B$12:$V$12</f>
             </numRef>
           </val>
         </ser>
@@ -551,12 +551,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$13:$U$13</f>
+              <f>'Data'!$B$13:$V$13</f>
             </numRef>
           </val>
         </ser>
@@ -583,12 +583,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$U$1</f>
+              <f>'Data'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$14:$U$14</f>
+              <f>'Data'!$B$14:$V$14</f>
             </numRef>
           </val>
         </ser>
@@ -975,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -999,6 +999,7 @@
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="7" customWidth="1" min="20" max="20"/>
     <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1067,6 +1068,9 @@
       <c r="U1" s="1" t="n">
         <v>95</v>
       </c>
+      <c r="V1" s="1" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1134,6 +1138,9 @@
       <c r="U2" t="n">
         <v>0.019</v>
       </c>
+      <c r="V2" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1201,6 +1208,9 @@
       <c r="U3" t="n">
         <v>0.015</v>
       </c>
+      <c r="V3" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1268,6 +1278,9 @@
       <c r="U4" t="n">
         <v>0.02</v>
       </c>
+      <c r="V4" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1335,6 +1348,9 @@
       <c r="U5" t="n">
         <v>0.044</v>
       </c>
+      <c r="V5" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1402,6 +1418,9 @@
       <c r="U6" t="n">
         <v>0.002</v>
       </c>
+      <c r="V6" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1469,6 +1488,9 @@
       <c r="U7" t="n">
         <v>0.012</v>
       </c>
+      <c r="V7" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1536,6 +1558,9 @@
       <c r="U8" t="n">
         <v>0.02</v>
       </c>
+      <c r="V8" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1603,6 +1628,9 @@
       <c r="U9" t="n">
         <v>0.002</v>
       </c>
+      <c r="V9" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1670,6 +1698,9 @@
       <c r="U10" t="n">
         <v>0</v>
       </c>
+      <c r="V10" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1737,6 +1768,9 @@
       <c r="U11" t="n">
         <v>0.008</v>
       </c>
+      <c r="V11" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1804,6 +1838,9 @@
       <c r="U12" t="n">
         <v>0</v>
       </c>
+      <c r="V12" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1871,6 +1908,9 @@
       <c r="U13" t="n">
         <v>0</v>
       </c>
+      <c r="V13" t="n">
+        <v>0.001</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1938,6 +1978,9 @@
       <c r="U14" t="n">
         <v>0.001</v>
       </c>
+      <c r="V14" t="n">
+        <v>0.001</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor all the codebase to be consistent and to work well with all the new methods TODO: test both ds
</commit_message>
<xml_diff>
--- a/results/excel_reports/resnet50_vgg16_black.xlsx
+++ b/results/excel_reports/resnet50_vgg16_black.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Top-1 Accuracy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Top-5 Accuracy" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -159,7 +160,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Accuracy Degradation</a:t>
+              <a:t>Top-1 Accuracy Degradation</a:t>
             </a:r>
           </a:p>
           <a:p>
@@ -181,7 +182,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Data'!A2</f>
+              <f>'Top-1 Accuracy'!A2</f>
             </strRef>
           </tx>
           <spPr>
@@ -199,12 +200,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$2:$V$2</f>
+              <f>'Top-1 Accuracy'!$B$2:$V$2</f>
             </numRef>
           </val>
         </ser>
@@ -213,7 +214,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Data'!A3</f>
+              <f>'Top-1 Accuracy'!A3</f>
             </strRef>
           </tx>
           <spPr>
@@ -231,12 +232,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$3:$V$3</f>
+              <f>'Top-1 Accuracy'!$B$3:$V$3</f>
             </numRef>
           </val>
         </ser>
@@ -245,7 +246,7 @@
           <order val="2"/>
           <tx>
             <strRef>
-              <f>'Data'!A4</f>
+              <f>'Top-1 Accuracy'!A4</f>
             </strRef>
           </tx>
           <spPr>
@@ -263,12 +264,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$4:$V$4</f>
+              <f>'Top-1 Accuracy'!$B$4:$V$4</f>
             </numRef>
           </val>
         </ser>
@@ -277,7 +278,7 @@
           <order val="3"/>
           <tx>
             <strRef>
-              <f>'Data'!A5</f>
+              <f>'Top-1 Accuracy'!A5</f>
             </strRef>
           </tx>
           <spPr>
@@ -295,12 +296,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$5:$V$5</f>
+              <f>'Top-1 Accuracy'!$B$5:$V$5</f>
             </numRef>
           </val>
         </ser>
@@ -309,7 +310,7 @@
           <order val="4"/>
           <tx>
             <strRef>
-              <f>'Data'!A6</f>
+              <f>'Top-1 Accuracy'!A6</f>
             </strRef>
           </tx>
           <spPr>
@@ -327,12 +328,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$6:$V$6</f>
+              <f>'Top-1 Accuracy'!$B$6:$V$6</f>
             </numRef>
           </val>
         </ser>
@@ -341,7 +342,7 @@
           <order val="5"/>
           <tx>
             <strRef>
-              <f>'Data'!A7</f>
+              <f>'Top-1 Accuracy'!A7</f>
             </strRef>
           </tx>
           <spPr>
@@ -359,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$7:$V$7</f>
+              <f>'Top-1 Accuracy'!$B$7:$V$7</f>
             </numRef>
           </val>
         </ser>
@@ -373,7 +374,7 @@
           <order val="6"/>
           <tx>
             <strRef>
-              <f>'Data'!A8</f>
+              <f>'Top-1 Accuracy'!A8</f>
             </strRef>
           </tx>
           <spPr>
@@ -391,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$8:$V$8</f>
+              <f>'Top-1 Accuracy'!$B$8:$V$8</f>
             </numRef>
           </val>
         </ser>
@@ -405,7 +406,7 @@
           <order val="7"/>
           <tx>
             <strRef>
-              <f>'Data'!A9</f>
+              <f>'Top-1 Accuracy'!A9</f>
             </strRef>
           </tx>
           <spPr>
@@ -423,140 +424,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Data'!$B$1:$V$1</f>
+              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Data'!$B$9:$V$9</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="8"/>
-          <order val="8"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A10</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$10:$V$10</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="9"/>
-          <order val="9"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A11</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$11:$V$11</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="10"/>
-          <order val="10"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A12</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$12:$V$12</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="11"/>
-          <order val="11"/>
-          <tx>
-            <strRef>
-              <f>'Data'!A13</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Data'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data'!$B$13:$V$13</f>
+              <f>'Top-1 Accuracy'!$B$9:$V$9</f>
             </numRef>
           </val>
         </ser>
@@ -627,13 +500,393 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Top-5 Accuracy Degradation</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Generator: resnet50 | Judge: vgg16 | Fill: black</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A2</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$2:$V$2</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$3:$V$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$4:$V$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$5:$V$5</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$6:$V$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A7</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$7:$V$7</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$8:$V$8</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <strRef>
+              <f>'Top-5 Accuracy'!A9</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Top-5 Accuracy'!$B$9:$V$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Occlusion Level (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.05"/>
+          <min val="0"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Top-5 Accuracy</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="tr"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9000000" cy="5400000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9000000" cy="5400000"/>
@@ -943,11 +1196,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1047,64 +1300,64 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C2" t="n">
-        <v>0.443</v>
+        <v>0.824</v>
       </c>
       <c r="D2" t="n">
-        <v>0.339</v>
+        <v>0.744</v>
       </c>
       <c r="E2" t="n">
-        <v>0.255</v>
+        <v>0.672</v>
       </c>
       <c r="F2" t="n">
-        <v>0.196</v>
+        <v>0.606</v>
       </c>
       <c r="G2" t="n">
-        <v>0.16</v>
+        <v>0.527</v>
       </c>
       <c r="H2" t="n">
-        <v>0.13</v>
+        <v>0.491</v>
       </c>
       <c r="I2" t="n">
+        <v>0.446</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.299</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.264</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="Q2" t="n">
         <v>0.099</v>
       </c>
-      <c r="J2" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.019</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.002</v>
-      </c>
       <c r="R2" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="U2" t="n">
         <v>0.001</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.002</v>
       </c>
       <c r="V2" t="n">
         <v>0.001</v>
@@ -1113,68 +1366,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gradientshap</t>
+          <t>integrated_gradients</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C3" t="n">
-        <v>0.485</v>
+        <v>0.843</v>
       </c>
       <c r="D3" t="n">
-        <v>0.356</v>
+        <v>0.779</v>
       </c>
       <c r="E3" t="n">
-        <v>0.275</v>
+        <v>0.712</v>
       </c>
       <c r="F3" t="n">
-        <v>0.23</v>
+        <v>0.661</v>
       </c>
       <c r="G3" t="n">
-        <v>0.185</v>
+        <v>0.59</v>
       </c>
       <c r="H3" t="n">
-        <v>0.154</v>
+        <v>0.543</v>
       </c>
       <c r="I3" t="n">
-        <v>0.125</v>
+        <v>0.483</v>
       </c>
       <c r="J3" t="n">
-        <v>0.1</v>
+        <v>0.446</v>
       </c>
       <c r="K3" t="n">
-        <v>0.079</v>
+        <v>0.4</v>
       </c>
       <c r="L3" t="n">
-        <v>0.063</v>
+        <v>0.362</v>
       </c>
       <c r="M3" t="n">
-        <v>0.047</v>
+        <v>0.315</v>
       </c>
       <c r="N3" t="n">
-        <v>0.025</v>
+        <v>0.263</v>
       </c>
       <c r="O3" t="n">
-        <v>0.017</v>
+        <v>0.241</v>
       </c>
       <c r="P3" t="n">
-        <v>0.01</v>
+        <v>0.191</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.004</v>
+        <v>0.132</v>
       </c>
       <c r="R3" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="U3" t="n">
         <v>0.006</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.003</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.002</v>
       </c>
       <c r="V3" t="n">
         <v>0.001</v>
@@ -1183,68 +1436,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>integrated_gradients</t>
+          <t>gradientshap</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C4" t="n">
-        <v>0.473</v>
+        <v>0.85</v>
       </c>
       <c r="D4" t="n">
-        <v>0.357</v>
+        <v>0.766</v>
       </c>
       <c r="E4" t="n">
-        <v>0.269</v>
+        <v>0.706</v>
       </c>
       <c r="F4" t="n">
-        <v>0.222</v>
+        <v>0.654</v>
       </c>
       <c r="G4" t="n">
-        <v>0.182</v>
+        <v>0.588</v>
       </c>
       <c r="H4" t="n">
-        <v>0.147</v>
+        <v>0.543</v>
       </c>
       <c r="I4" t="n">
-        <v>0.12</v>
+        <v>0.498</v>
       </c>
       <c r="J4" t="n">
-        <v>0.106</v>
+        <v>0.442</v>
       </c>
       <c r="K4" t="n">
-        <v>0.075</v>
+        <v>0.398</v>
       </c>
       <c r="L4" t="n">
-        <v>0.058</v>
+        <v>0.35</v>
       </c>
       <c r="M4" t="n">
-        <v>0.038</v>
+        <v>0.307</v>
       </c>
       <c r="N4" t="n">
-        <v>0.034</v>
+        <v>0.265</v>
       </c>
       <c r="O4" t="n">
-        <v>0.025</v>
+        <v>0.214</v>
       </c>
       <c r="P4" t="n">
-        <v>0.015</v>
+        <v>0.176</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.008</v>
+        <v>0.135</v>
       </c>
       <c r="R4" t="n">
-        <v>0.003</v>
+        <v>0.093</v>
       </c>
       <c r="S4" t="n">
-        <v>0.003</v>
+        <v>0.06</v>
       </c>
       <c r="T4" t="n">
-        <v>0.002</v>
+        <v>0.03</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="V4" t="n">
         <v>0.001</v>
@@ -1253,138 +1506,138 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>inputxgradient_continuous</t>
+          <t>saliency</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C5" t="n">
-        <v>0.721</v>
+        <v>0.854</v>
       </c>
       <c r="D5" t="n">
-        <v>0.636</v>
+        <v>0.782</v>
       </c>
       <c r="E5" t="n">
-        <v>0.538</v>
+        <v>0.731</v>
       </c>
       <c r="F5" t="n">
-        <v>0.485</v>
+        <v>0.644</v>
       </c>
       <c r="G5" t="n">
-        <v>0.417</v>
+        <v>0.585</v>
       </c>
       <c r="H5" t="n">
-        <v>0.35</v>
+        <v>0.527</v>
       </c>
       <c r="I5" t="n">
-        <v>0.298</v>
+        <v>0.466</v>
       </c>
       <c r="J5" t="n">
-        <v>0.257</v>
+        <v>0.42</v>
       </c>
       <c r="K5" t="n">
-        <v>0.224</v>
+        <v>0.379</v>
       </c>
       <c r="L5" t="n">
-        <v>0.171</v>
+        <v>0.339</v>
       </c>
       <c r="M5" t="n">
-        <v>0.138</v>
+        <v>0.297</v>
       </c>
       <c r="N5" t="n">
-        <v>0.106</v>
+        <v>0.259</v>
       </c>
       <c r="O5" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.216</v>
       </c>
       <c r="P5" t="n">
-        <v>0.062</v>
+        <v>0.178</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.038</v>
+        <v>0.149</v>
       </c>
       <c r="R5" t="n">
-        <v>0.027</v>
+        <v>0.123</v>
       </c>
       <c r="S5" t="n">
-        <v>0.011</v>
+        <v>0.105</v>
       </c>
       <c r="T5" t="n">
-        <v>0.004</v>
+        <v>0.092</v>
       </c>
       <c r="U5" t="n">
-        <v>0.003</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="V5" t="n">
-        <v>0.001</v>
+        <v>0.082</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>xrai</t>
+          <t>guided_backprop</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C6" t="n">
-        <v>0.706</v>
+        <v>0.883</v>
       </c>
       <c r="D6" t="n">
-        <v>0.607</v>
+        <v>0.842</v>
       </c>
       <c r="E6" t="n">
-        <v>0.543</v>
+        <v>0.803</v>
       </c>
       <c r="F6" t="n">
-        <v>0.473</v>
+        <v>0.757</v>
       </c>
       <c r="G6" t="n">
-        <v>0.418</v>
+        <v>0.727</v>
       </c>
       <c r="H6" t="n">
-        <v>0.358</v>
+        <v>0.676</v>
       </c>
       <c r="I6" t="n">
-        <v>0.314</v>
+        <v>0.636</v>
       </c>
       <c r="J6" t="n">
-        <v>0.267</v>
+        <v>0.594</v>
       </c>
       <c r="K6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.461</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.428</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.294</v>
+      </c>
+      <c r="S6" t="n">
         <v>0.229</v>
       </c>
-      <c r="L6" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.164</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="O6" t="n">
+      <c r="T6" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="U6" t="n">
         <v>0.101</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="T6" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0.001</v>
       </c>
       <c r="V6" t="n">
         <v>0.001</v>
@@ -1393,68 +1646,68 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>guided_backprop</t>
+          <t>xrai</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C7" t="n">
-        <v>0.576</v>
+        <v>0.914</v>
       </c>
       <c r="D7" t="n">
-        <v>0.501</v>
+        <v>0.9</v>
       </c>
       <c r="E7" t="n">
-        <v>0.44</v>
+        <v>0.884</v>
       </c>
       <c r="F7" t="n">
-        <v>0.39</v>
+        <v>0.861</v>
       </c>
       <c r="G7" t="n">
-        <v>0.347</v>
+        <v>0.855</v>
       </c>
       <c r="H7" t="n">
-        <v>0.315</v>
+        <v>0.827</v>
       </c>
       <c r="I7" t="n">
-        <v>0.278</v>
+        <v>0.789</v>
       </c>
       <c r="J7" t="n">
-        <v>0.244</v>
+        <v>0.753</v>
       </c>
       <c r="K7" t="n">
-        <v>0.218</v>
+        <v>0.728</v>
       </c>
       <c r="L7" t="n">
-        <v>0.19</v>
+        <v>0.675</v>
       </c>
       <c r="M7" t="n">
-        <v>0.173</v>
+        <v>0.636</v>
       </c>
       <c r="N7" t="n">
-        <v>0.146</v>
+        <v>0.573</v>
       </c>
       <c r="O7" t="n">
-        <v>0.122</v>
+        <v>0.529</v>
       </c>
       <c r="P7" t="n">
-        <v>0.098</v>
+        <v>0.45</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.398</v>
       </c>
       <c r="R7" t="n">
-        <v>0.059</v>
+        <v>0.306</v>
       </c>
       <c r="S7" t="n">
-        <v>0.039</v>
+        <v>0.239</v>
       </c>
       <c r="T7" t="n">
-        <v>0.022</v>
+        <v>0.135</v>
       </c>
       <c r="U7" t="n">
-        <v>0.012</v>
+        <v>0.042</v>
       </c>
       <c r="V7" t="n">
         <v>0.001</v>
@@ -1463,68 +1716,68 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>occlusion</t>
+          <t>grad_cam</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.829</v>
+        <v>0.9199199199199199</v>
       </c>
       <c r="C8" t="n">
-        <v>0.622</v>
+        <v>0.892</v>
       </c>
       <c r="D8" t="n">
-        <v>0.519</v>
+        <v>0.888</v>
       </c>
       <c r="E8" t="n">
-        <v>0.425</v>
+        <v>0.875</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4</v>
+        <v>0.857</v>
       </c>
       <c r="G8" t="n">
-        <v>0.352</v>
+        <v>0.855</v>
       </c>
       <c r="H8" t="n">
-        <v>0.311</v>
+        <v>0.836</v>
       </c>
       <c r="I8" t="n">
-        <v>0.281</v>
+        <v>0.827</v>
       </c>
       <c r="J8" t="n">
-        <v>0.256</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>0.222</v>
+        <v>0.794</v>
       </c>
       <c r="L8" t="n">
-        <v>0.201</v>
+        <v>0.779</v>
       </c>
       <c r="M8" t="n">
-        <v>0.183</v>
+        <v>0.748</v>
       </c>
       <c r="N8" t="n">
-        <v>0.146</v>
+        <v>0.724</v>
       </c>
       <c r="O8" t="n">
-        <v>0.129</v>
+        <v>0.697</v>
       </c>
       <c r="P8" t="n">
-        <v>0.105</v>
+        <v>0.673</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.089</v>
+        <v>0.625</v>
       </c>
       <c r="R8" t="n">
-        <v>0.064</v>
+        <v>0.571</v>
       </c>
       <c r="S8" t="n">
-        <v>0.041</v>
+        <v>0.503</v>
       </c>
       <c r="T8" t="n">
-        <v>0.021</v>
+        <v>0.371</v>
       </c>
       <c r="U8" t="n">
-        <v>0.008</v>
+        <v>0.199</v>
       </c>
       <c r="V8" t="n">
         <v>0.001</v>
@@ -1533,355 +1786,756 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>guided_gradcam</t>
+          <t>occlusion</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>0.9199199199199199</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.851</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="P9" t="n">
         <v>0.829</v>
       </c>
-      <c r="C9" t="n">
+      <c r="Q9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="S9" t="n">
         <v>0.714</v>
       </c>
-      <c r="D9" t="n">
-        <v>0.648</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.602</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.544</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.457</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.425</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.386</v>
-      </c>
-      <c r="K9" t="n">
+      <c r="T9" t="n">
+        <v>0.618</v>
+      </c>
+      <c r="U9" t="n">
         <v>0.346</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.197</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.166</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.095</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.039</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0.02</v>
       </c>
       <c r="V9" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+  </sheetData>
+  <conditionalFormatting sqref="B2:V9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.5"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>dinov2_attention</t>
+          <t>attribution_method</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.645</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.611</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.572</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.527</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.422</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.377</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.328</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.307</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.281</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0.195</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0.141</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0.044</v>
-      </c>
-      <c r="U10" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0.001</v>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="H1" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="I1" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="J1" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="K1" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="L1" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="M1" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="N1" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="O1" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="P1" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q1" s="1" t="n">
+        <v>75</v>
+      </c>
+      <c r="R1" s="1" t="n">
+        <v>80</v>
+      </c>
+      <c r="S1" s="1" t="n">
+        <v>85</v>
+      </c>
+      <c r="T1" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="U1" s="1" t="n">
+        <v>95</v>
+      </c>
+      <c r="V1" s="1" t="n">
+        <v>100</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
-          <t>dinov2_PC1</t>
+          <t>inputxgradient</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.757</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.723</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.709</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0.647</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.617</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.586</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.487</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.426</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.376</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.324</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0.276</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0.229</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.171</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0.106</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0.064</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0.029</v>
-      </c>
-      <c r="U11" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0.001</v>
+      <c r="B2" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.697</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.379</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.316</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.253</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.198</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.005</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
-          <t>dinov2_COMBO_FIXED</t>
+          <t>saliency</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.758</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.721</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.702</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.661</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0.653</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.614</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.574</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0.473</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.412</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0.365</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.278</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0.235</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0.038</v>
-      </c>
-      <c r="U12" t="n">
-        <v>0.011</v>
-      </c>
-      <c r="V12" t="n">
-        <v>0.001</v>
+      <c r="B3" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.696</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.542</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.438</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.267</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.219</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.182</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0.09</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
-          <t>inputxgradient_u2net_fill</t>
+          <t>gradientshap</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.6820000000000001</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.621</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.586</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.532</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.518</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0.466</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.434</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.378</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.335</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0.311</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0.264</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0.203</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0.148</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0.028</v>
-      </c>
-      <c r="V13" t="n">
-        <v>0.001</v>
+      <c r="B4" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.879</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.745</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.644</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.484</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.327</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.188</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>integrated_gradients</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.747</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>guided_backprop</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.909</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.666</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.594</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0.496</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="V6" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>xrai</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.968</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.714</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.578</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0.103</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>grad_cam</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.914</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.866</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.819</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0.5659999999999999</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>occlusion</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.98998998998999</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.983</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.929</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.554</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.005</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:V13">
+  <conditionalFormatting sqref="B2:V9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
added the second sipak model
</commit_message>
<xml_diff>
--- a/results/excel_reports/resnet50_vgg16_black.xlsx
+++ b/results/excel_reports/resnet50_vgg16_black.xlsx
@@ -369,70 +369,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <strRef>
-              <f>'Top-1 Accuracy'!A8</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Top-1 Accuracy'!$B$8:$V$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <tx>
-            <strRef>
-              <f>'Top-1 Accuracy'!A9</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Top-1 Accuracy'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Top-1 Accuracy'!$B$9:$V$9</f>
-            </numRef>
-          </val>
-        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -722,70 +658,6 @@
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <strRef>
-              <f>'Top-5 Accuracy'!A8</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Top-5 Accuracy'!$B$8:$V$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
-          <tx>
-            <strRef>
-              <f>'Top-5 Accuracy'!A9</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Top-5 Accuracy'!$B$1:$V$1</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Top-5 Accuracy'!$B$9:$V$9</f>
-            </numRef>
-          </val>
-        </ser>
         <axId val="10"/>
         <axId val="100"/>
       </lineChart>
@@ -859,7 +731,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9000000" cy="5400000"/>
@@ -886,7 +758,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>9</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="9000000" cy="5400000"/>
@@ -1196,11 +1068,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1296,68 +1168,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>inputxgradient</t>
+          <t>gradientshap</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.824</v>
+        <v>0.387</v>
       </c>
       <c r="D2" t="n">
-        <v>0.744</v>
+        <v>0.252</v>
       </c>
       <c r="E2" t="n">
-        <v>0.672</v>
+        <v>0.187</v>
       </c>
       <c r="F2" t="n">
-        <v>0.606</v>
+        <v>0.147</v>
       </c>
       <c r="G2" t="n">
-        <v>0.527</v>
+        <v>0.115</v>
       </c>
       <c r="H2" t="n">
-        <v>0.491</v>
+        <v>0.093</v>
       </c>
       <c r="I2" t="n">
-        <v>0.446</v>
+        <v>0.064</v>
       </c>
       <c r="J2" t="n">
-        <v>0.402</v>
+        <v>0.05</v>
       </c>
       <c r="K2" t="n">
-        <v>0.345</v>
+        <v>0.032</v>
       </c>
       <c r="L2" t="n">
-        <v>0.299</v>
+        <v>0.019</v>
       </c>
       <c r="M2" t="n">
-        <v>0.264</v>
+        <v>0.012</v>
       </c>
       <c r="N2" t="n">
-        <v>0.213</v>
+        <v>0.01</v>
       </c>
       <c r="O2" t="n">
-        <v>0.178</v>
+        <v>0.01</v>
       </c>
       <c r="P2" t="n">
-        <v>0.133</v>
+        <v>0.004</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.099</v>
+        <v>0.002</v>
       </c>
       <c r="R2" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>0.04</v>
+        <v>0.002</v>
       </c>
       <c r="T2" t="n">
-        <v>0.014</v>
+        <v>0.001</v>
       </c>
       <c r="U2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="V2" t="n">
         <v>0.001</v>
@@ -1366,68 +1238,68 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>integrated_gradients</t>
+          <t>inputxgradient</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>0.843</v>
+        <v>0.357</v>
       </c>
       <c r="D3" t="n">
-        <v>0.779</v>
+        <v>0.218</v>
       </c>
       <c r="E3" t="n">
-        <v>0.712</v>
+        <v>0.157</v>
       </c>
       <c r="F3" t="n">
-        <v>0.661</v>
+        <v>0.118</v>
       </c>
       <c r="G3" t="n">
-        <v>0.59</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>0.543</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>0.483</v>
+        <v>0.055</v>
       </c>
       <c r="J3" t="n">
-        <v>0.446</v>
+        <v>0.043</v>
       </c>
       <c r="K3" t="n">
-        <v>0.4</v>
+        <v>0.022</v>
       </c>
       <c r="L3" t="n">
-        <v>0.362</v>
+        <v>0.015</v>
       </c>
       <c r="M3" t="n">
-        <v>0.315</v>
+        <v>0.007</v>
       </c>
       <c r="N3" t="n">
-        <v>0.263</v>
+        <v>0.003</v>
       </c>
       <c r="O3" t="n">
-        <v>0.241</v>
+        <v>0.002</v>
       </c>
       <c r="P3" t="n">
-        <v>0.191</v>
+        <v>0.002</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.132</v>
+        <v>0.002</v>
       </c>
       <c r="R3" t="n">
-        <v>0.101</v>
+        <v>0.002</v>
       </c>
       <c r="S3" t="n">
-        <v>0.064</v>
+        <v>0.001</v>
       </c>
       <c r="T3" t="n">
-        <v>0.029</v>
+        <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
       <c r="V3" t="n">
         <v>0.001</v>
@@ -1436,68 +1308,68 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gradientshap</t>
+          <t>integrated_gradients</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>0.85</v>
+        <v>0.391</v>
       </c>
       <c r="D4" t="n">
-        <v>0.766</v>
+        <v>0.248</v>
       </c>
       <c r="E4" t="n">
-        <v>0.706</v>
+        <v>0.195</v>
       </c>
       <c r="F4" t="n">
-        <v>0.654</v>
+        <v>0.157</v>
       </c>
       <c r="G4" t="n">
-        <v>0.588</v>
+        <v>0.121</v>
       </c>
       <c r="H4" t="n">
-        <v>0.543</v>
+        <v>0.091</v>
       </c>
       <c r="I4" t="n">
-        <v>0.498</v>
+        <v>0.075</v>
       </c>
       <c r="J4" t="n">
-        <v>0.442</v>
+        <v>0.045</v>
       </c>
       <c r="K4" t="n">
-        <v>0.398</v>
+        <v>0.041</v>
       </c>
       <c r="L4" t="n">
-        <v>0.35</v>
+        <v>0.03</v>
       </c>
       <c r="M4" t="n">
-        <v>0.307</v>
+        <v>0.013</v>
       </c>
       <c r="N4" t="n">
-        <v>0.265</v>
+        <v>0.007</v>
       </c>
       <c r="O4" t="n">
-        <v>0.214</v>
+        <v>0.007</v>
       </c>
       <c r="P4" t="n">
-        <v>0.176</v>
+        <v>0.003</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.135</v>
+        <v>0.002</v>
       </c>
       <c r="R4" t="n">
-        <v>0.093</v>
+        <v>0.001</v>
       </c>
       <c r="S4" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.03</v>
+        <v>0.001</v>
       </c>
       <c r="U4" t="n">
-        <v>0.013</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
         <v>0.001</v>
@@ -1510,134 +1382,134 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.854</v>
+        <v>0.34</v>
       </c>
       <c r="D5" t="n">
-        <v>0.782</v>
+        <v>0.223</v>
       </c>
       <c r="E5" t="n">
-        <v>0.731</v>
+        <v>0.164</v>
       </c>
       <c r="F5" t="n">
-        <v>0.644</v>
+        <v>0.101</v>
       </c>
       <c r="G5" t="n">
-        <v>0.585</v>
+        <v>0.081</v>
       </c>
       <c r="H5" t="n">
-        <v>0.527</v>
+        <v>0.063</v>
       </c>
       <c r="I5" t="n">
-        <v>0.466</v>
+        <v>0.045</v>
       </c>
       <c r="J5" t="n">
-        <v>0.42</v>
+        <v>0.028</v>
       </c>
       <c r="K5" t="n">
-        <v>0.379</v>
+        <v>0.02</v>
       </c>
       <c r="L5" t="n">
-        <v>0.339</v>
+        <v>0.006</v>
       </c>
       <c r="M5" t="n">
-        <v>0.297</v>
+        <v>0.007</v>
       </c>
       <c r="N5" t="n">
-        <v>0.259</v>
+        <v>0.004</v>
       </c>
       <c r="O5" t="n">
-        <v>0.216</v>
+        <v>0.003</v>
       </c>
       <c r="P5" t="n">
-        <v>0.178</v>
+        <v>0.003</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.149</v>
+        <v>0.002</v>
       </c>
       <c r="R5" t="n">
-        <v>0.123</v>
+        <v>0.002</v>
       </c>
       <c r="S5" t="n">
-        <v>0.105</v>
+        <v>0.001</v>
       </c>
       <c r="T5" t="n">
-        <v>0.092</v>
+        <v>0.001</v>
       </c>
       <c r="U5" t="n">
-        <v>0.08500000000000001</v>
+        <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>0.082</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>guided_backprop</t>
+          <t>smoothgrad</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>0.883</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>0.842</v>
+        <v>0.578</v>
       </c>
       <c r="E6" t="n">
-        <v>0.803</v>
+        <v>0.486</v>
       </c>
       <c r="F6" t="n">
-        <v>0.757</v>
+        <v>0.424</v>
       </c>
       <c r="G6" t="n">
-        <v>0.727</v>
+        <v>0.362</v>
       </c>
       <c r="H6" t="n">
-        <v>0.676</v>
+        <v>0.297</v>
       </c>
       <c r="I6" t="n">
-        <v>0.636</v>
+        <v>0.234</v>
       </c>
       <c r="J6" t="n">
-        <v>0.594</v>
+        <v>0.185</v>
       </c>
       <c r="K6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.151</v>
       </c>
       <c r="L6" t="n">
-        <v>0.52</v>
+        <v>0.111</v>
       </c>
       <c r="M6" t="n">
-        <v>0.496</v>
+        <v>0.076</v>
       </c>
       <c r="N6" t="n">
-        <v>0.461</v>
+        <v>0.061</v>
       </c>
       <c r="O6" t="n">
-        <v>0.428</v>
+        <v>0.041</v>
       </c>
       <c r="P6" t="n">
-        <v>0.384</v>
+        <v>0.026</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.336</v>
+        <v>0.017</v>
       </c>
       <c r="R6" t="n">
-        <v>0.294</v>
+        <v>0.008</v>
       </c>
       <c r="S6" t="n">
-        <v>0.229</v>
+        <v>0.003</v>
       </c>
       <c r="T6" t="n">
-        <v>0.171</v>
+        <v>0.002</v>
       </c>
       <c r="U6" t="n">
-        <v>0.101</v>
+        <v>0.001</v>
       </c>
       <c r="V6" t="n">
         <v>0.001</v>
@@ -1646,215 +1518,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>xrai</t>
+          <t>grad_cam</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.9199199199199199</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>0.914</v>
+        <v>0.78</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9</v>
+        <v>0.756</v>
       </c>
       <c r="E7" t="n">
-        <v>0.884</v>
+        <v>0.734</v>
       </c>
       <c r="F7" t="n">
-        <v>0.861</v>
+        <v>0.71</v>
       </c>
       <c r="G7" t="n">
-        <v>0.855</v>
+        <v>0.709</v>
       </c>
       <c r="H7" t="n">
-        <v>0.827</v>
+        <v>0.705</v>
       </c>
       <c r="I7" t="n">
-        <v>0.789</v>
+        <v>0.68</v>
       </c>
       <c r="J7" t="n">
-        <v>0.753</v>
+        <v>0.64</v>
       </c>
       <c r="K7" t="n">
-        <v>0.728</v>
+        <v>0.621</v>
       </c>
       <c r="L7" t="n">
-        <v>0.675</v>
+        <v>0.601</v>
       </c>
       <c r="M7" t="n">
-        <v>0.636</v>
+        <v>0.556</v>
       </c>
       <c r="N7" t="n">
-        <v>0.573</v>
+        <v>0.516</v>
       </c>
       <c r="O7" t="n">
-        <v>0.529</v>
+        <v>0.479</v>
       </c>
       <c r="P7" t="n">
-        <v>0.45</v>
+        <v>0.427</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.398</v>
+        <v>0.397</v>
       </c>
       <c r="R7" t="n">
-        <v>0.306</v>
+        <v>0.294</v>
       </c>
       <c r="S7" t="n">
-        <v>0.239</v>
+        <v>0.224</v>
       </c>
       <c r="T7" t="n">
-        <v>0.135</v>
+        <v>0.114</v>
       </c>
       <c r="U7" t="n">
-        <v>0.042</v>
+        <v>0.032</v>
       </c>
       <c r="V7" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>grad_cam</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.9199199199199199</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.892</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.888</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.857</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.855</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.836</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.827</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.8070000000000001</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.779</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.748</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.724</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.697</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.673</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.571</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.371</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.199</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>occlusion</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.9199199199199199</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.918</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.888</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.887</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.887</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.872</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.856</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.851</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.842</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.775</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.618</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0.346</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0.001</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:V9">
+  <conditionalFormatting sqref="B2:V7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -1877,11 +1609,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1981,64 +1713,64 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C2" t="n">
-        <v>0.955</v>
+        <v>0.585</v>
       </c>
       <c r="D2" t="n">
-        <v>0.905</v>
+        <v>0.412</v>
       </c>
       <c r="E2" t="n">
-        <v>0.85</v>
+        <v>0.33</v>
       </c>
       <c r="F2" t="n">
-        <v>0.794</v>
+        <v>0.254</v>
       </c>
       <c r="G2" t="n">
-        <v>0.748</v>
+        <v>0.205</v>
       </c>
       <c r="H2" t="n">
-        <v>0.697</v>
+        <v>0.165</v>
       </c>
       <c r="I2" t="n">
-        <v>0.65</v>
+        <v>0.129</v>
       </c>
       <c r="J2" t="n">
-        <v>0.598</v>
+        <v>0.103</v>
       </c>
       <c r="K2" t="n">
-        <v>0.54</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="L2" t="n">
-        <v>0.483</v>
+        <v>0.05</v>
       </c>
       <c r="M2" t="n">
-        <v>0.42</v>
+        <v>0.036</v>
       </c>
       <c r="N2" t="n">
-        <v>0.379</v>
+        <v>0.023</v>
       </c>
       <c r="O2" t="n">
-        <v>0.316</v>
+        <v>0.018</v>
       </c>
       <c r="P2" t="n">
-        <v>0.253</v>
+        <v>0.014</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.198</v>
+        <v>0.01</v>
       </c>
       <c r="R2" t="n">
-        <v>0.135</v>
+        <v>0.006</v>
       </c>
       <c r="S2" t="n">
-        <v>0.094</v>
+        <v>0.006</v>
       </c>
       <c r="T2" t="n">
-        <v>0.032</v>
+        <v>0.007</v>
       </c>
       <c r="U2" t="n">
-        <v>0.014</v>
+        <v>0.006</v>
       </c>
       <c r="V2" t="n">
         <v>0.005</v>
@@ -2051,134 +1783,134 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C3" t="n">
-        <v>0.958</v>
+        <v>0.569</v>
       </c>
       <c r="D3" t="n">
-        <v>0.912</v>
+        <v>0.408</v>
       </c>
       <c r="E3" t="n">
-        <v>0.862</v>
+        <v>0.334</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8110000000000001</v>
+        <v>0.256</v>
       </c>
       <c r="G3" t="n">
-        <v>0.754</v>
+        <v>0.204</v>
       </c>
       <c r="H3" t="n">
-        <v>0.696</v>
+        <v>0.157</v>
       </c>
       <c r="I3" t="n">
-        <v>0.638</v>
+        <v>0.124</v>
       </c>
       <c r="J3" t="n">
-        <v>0.578</v>
+        <v>0.093</v>
       </c>
       <c r="K3" t="n">
-        <v>0.542</v>
+        <v>0.078</v>
       </c>
       <c r="L3" t="n">
-        <v>0.484</v>
+        <v>0.052</v>
       </c>
       <c r="M3" t="n">
-        <v>0.438</v>
+        <v>0.038</v>
       </c>
       <c r="N3" t="n">
-        <v>0.386</v>
+        <v>0.028</v>
       </c>
       <c r="O3" t="n">
-        <v>0.322</v>
+        <v>0.025</v>
       </c>
       <c r="P3" t="n">
-        <v>0.267</v>
+        <v>0.02</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.219</v>
+        <v>0.01</v>
       </c>
       <c r="R3" t="n">
-        <v>0.182</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>0.142</v>
+        <v>0.004</v>
       </c>
       <c r="T3" t="n">
-        <v>0.112</v>
+        <v>0.004</v>
       </c>
       <c r="U3" t="n">
-        <v>0.096</v>
+        <v>0.005</v>
       </c>
       <c r="V3" t="n">
-        <v>0.09</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gradientshap</t>
+          <t>integrated_gradients</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C4" t="n">
-        <v>0.965</v>
+        <v>0.632</v>
       </c>
       <c r="D4" t="n">
-        <v>0.925</v>
+        <v>0.476</v>
       </c>
       <c r="E4" t="n">
-        <v>0.879</v>
+        <v>0.372</v>
       </c>
       <c r="F4" t="n">
-        <v>0.833</v>
+        <v>0.297</v>
       </c>
       <c r="G4" t="n">
-        <v>0.778</v>
+        <v>0.254</v>
       </c>
       <c r="H4" t="n">
-        <v>0.745</v>
+        <v>0.207</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.163</v>
       </c>
       <c r="J4" t="n">
-        <v>0.644</v>
+        <v>0.136</v>
       </c>
       <c r="K4" t="n">
-        <v>0.588</v>
+        <v>0.097</v>
       </c>
       <c r="L4" t="n">
-        <v>0.536</v>
+        <v>0.078</v>
       </c>
       <c r="M4" t="n">
-        <v>0.484</v>
+        <v>0.062</v>
       </c>
       <c r="N4" t="n">
-        <v>0.452</v>
+        <v>0.037</v>
       </c>
       <c r="O4" t="n">
-        <v>0.392</v>
+        <v>0.029</v>
       </c>
       <c r="P4" t="n">
-        <v>0.327</v>
+        <v>0.017</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.256</v>
+        <v>0.015</v>
       </c>
       <c r="R4" t="n">
-        <v>0.188</v>
+        <v>0.012</v>
       </c>
       <c r="S4" t="n">
-        <v>0.139</v>
+        <v>0.007</v>
       </c>
       <c r="T4" t="n">
-        <v>0.068</v>
+        <v>0.006</v>
       </c>
       <c r="U4" t="n">
-        <v>0.03</v>
+        <v>0.006</v>
       </c>
       <c r="V4" t="n">
         <v>0.005</v>
@@ -2187,68 +1919,68 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>integrated_gradients</t>
+          <t>gradientshap</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C5" t="n">
-        <v>0.965</v>
+        <v>0.628</v>
       </c>
       <c r="D5" t="n">
-        <v>0.929</v>
+        <v>0.463</v>
       </c>
       <c r="E5" t="n">
-        <v>0.868</v>
+        <v>0.365</v>
       </c>
       <c r="F5" t="n">
-        <v>0.83</v>
+        <v>0.282</v>
       </c>
       <c r="G5" t="n">
-        <v>0.784</v>
+        <v>0.246</v>
       </c>
       <c r="H5" t="n">
-        <v>0.747</v>
+        <v>0.199</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.155</v>
       </c>
       <c r="J5" t="n">
-        <v>0.655</v>
+        <v>0.131</v>
       </c>
       <c r="K5" t="n">
-        <v>0.597</v>
+        <v>0.095</v>
       </c>
       <c r="L5" t="n">
-        <v>0.554</v>
+        <v>0.074</v>
       </c>
       <c r="M5" t="n">
-        <v>0.496</v>
+        <v>0.06</v>
       </c>
       <c r="N5" t="n">
-        <v>0.441</v>
+        <v>0.039</v>
       </c>
       <c r="O5" t="n">
-        <v>0.391</v>
+        <v>0.027</v>
       </c>
       <c r="P5" t="n">
-        <v>0.33</v>
+        <v>0.025</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.27</v>
+        <v>0.019</v>
       </c>
       <c r="R5" t="n">
-        <v>0.19</v>
+        <v>0.01</v>
       </c>
       <c r="S5" t="n">
-        <v>0.144</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="T5" t="n">
-        <v>0.079</v>
+        <v>0.005</v>
       </c>
       <c r="U5" t="n">
-        <v>0.025</v>
+        <v>0.005</v>
       </c>
       <c r="V5" t="n">
         <v>0.005</v>
@@ -2257,68 +1989,68 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>guided_backprop</t>
+          <t>smoothgrad</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C6" t="n">
-        <v>0.979</v>
+        <v>0.888</v>
       </c>
       <c r="D6" t="n">
-        <v>0.952</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="E6" t="n">
-        <v>0.929</v>
+        <v>0.709</v>
       </c>
       <c r="F6" t="n">
-        <v>0.909</v>
+        <v>0.642</v>
       </c>
       <c r="G6" t="n">
-        <v>0.88</v>
+        <v>0.58</v>
       </c>
       <c r="H6" t="n">
-        <v>0.858</v>
+        <v>0.504</v>
       </c>
       <c r="I6" t="n">
-        <v>0.828</v>
+        <v>0.432</v>
       </c>
       <c r="J6" t="n">
-        <v>0.798</v>
+        <v>0.368</v>
       </c>
       <c r="K6" t="n">
-        <v>0.754</v>
+        <v>0.308</v>
       </c>
       <c r="L6" t="n">
-        <v>0.732</v>
+        <v>0.251</v>
       </c>
       <c r="M6" t="n">
-        <v>0.712</v>
+        <v>0.208</v>
       </c>
       <c r="N6" t="n">
-        <v>0.666</v>
+        <v>0.166</v>
       </c>
       <c r="O6" t="n">
-        <v>0.625</v>
+        <v>0.115</v>
       </c>
       <c r="P6" t="n">
-        <v>0.594</v>
+        <v>0.082</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.552</v>
+        <v>0.053</v>
       </c>
       <c r="R6" t="n">
-        <v>0.496</v>
+        <v>0.039</v>
       </c>
       <c r="S6" t="n">
-        <v>0.43</v>
+        <v>0.023</v>
       </c>
       <c r="T6" t="n">
-        <v>0.339</v>
+        <v>0.011</v>
       </c>
       <c r="U6" t="n">
-        <v>0.21</v>
+        <v>0.006</v>
       </c>
       <c r="V6" t="n">
         <v>0.005</v>
@@ -2327,215 +2059,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>xrai</t>
+          <t>grad_cam</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.98998998998999</v>
+        <v>0.952</v>
       </c>
       <c r="C7" t="n">
-        <v>0.985</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>0.98</v>
+        <v>0.92</v>
       </c>
       <c r="E7" t="n">
-        <v>0.973</v>
+        <v>0.916</v>
       </c>
       <c r="F7" t="n">
-        <v>0.968</v>
+        <v>0.908</v>
       </c>
       <c r="G7" t="n">
-        <v>0.967</v>
+        <v>0.902</v>
       </c>
       <c r="H7" t="n">
-        <v>0.949</v>
+        <v>0.897</v>
       </c>
       <c r="I7" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.887</v>
       </c>
       <c r="J7" t="n">
-        <v>0.912</v>
+        <v>0.869</v>
       </c>
       <c r="K7" t="n">
-        <v>0.894</v>
+        <v>0.842</v>
       </c>
       <c r="L7" t="n">
-        <v>0.848</v>
+        <v>0.821</v>
       </c>
       <c r="M7" t="n">
-        <v>0.805</v>
+        <v>0.792</v>
       </c>
       <c r="N7" t="n">
-        <v>0.764</v>
+        <v>0.753</v>
       </c>
       <c r="O7" t="n">
-        <v>0.714</v>
+        <v>0.695</v>
       </c>
       <c r="P7" t="n">
-        <v>0.641</v>
+        <v>0.663</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.578</v>
+        <v>0.587</v>
       </c>
       <c r="R7" t="n">
-        <v>0.468</v>
+        <v>0.502</v>
       </c>
       <c r="S7" t="n">
-        <v>0.373</v>
+        <v>0.38</v>
       </c>
       <c r="T7" t="n">
-        <v>0.245</v>
+        <v>0.249</v>
       </c>
       <c r="U7" t="n">
-        <v>0.103</v>
+        <v>0.098</v>
       </c>
       <c r="V7" t="n">
         <v>0.005</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>grad_cam</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.98998998998999</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.978</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.967</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.965</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.959</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.947</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.929</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.925</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.914</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.866</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.841</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0.819</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0.766</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0.5659999999999999</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0.361</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>occlusion</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.98998998998999</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.983</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.979</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.967</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.963</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.957</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0.929</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0.911</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0.872</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0.792</v>
-      </c>
-      <c r="U9" t="n">
-        <v>0.554</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0.005</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:V9">
+  <conditionalFormatting sqref="B2:V7">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>